<commit_message>
Complete demo seed setup
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="147">
   <si>
     <t>okul_no</t>
   </si>
@@ -62,10 +62,10 @@
     <t>100</t>
   </si>
   <si>
-    <t>Ogrenci</t>
-  </si>
-  <si>
-    <t>Deneme</t>
+    <t>Veli</t>
+  </si>
+  <si>
+    <t>Yaşar</t>
   </si>
   <si>
     <t>8-A</t>
@@ -80,7 +80,7 @@
     <t>5550000014</t>
   </si>
   <si>
-    <t>Veli</t>
+    <t>Dilber</t>
   </si>
   <si>
     <t>5550000001</t>
@@ -89,10 +89,7 @@
     <t>veli@example.com</t>
   </si>
   <si>
-    <t>hayir</t>
-  </si>
-  <si>
-    <t>evet</t>
+    <t>Evet</t>
   </si>
   <si>
     <t>101</t>
@@ -104,25 +101,340 @@
     <t>Kaya</t>
   </si>
   <si>
+    <t>ali.kaya@example.com</t>
+  </si>
+  <si>
+    <t>10000001372</t>
+  </si>
+  <si>
+    <t>5550000015</t>
+  </si>
+  <si>
+    <t>Mehmet</t>
+  </si>
+  <si>
+    <t>5550000002</t>
+  </si>
+  <si>
+    <t>veli.kaya@example.com</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>Ahmet</t>
+  </si>
+  <si>
+    <t>Saya</t>
+  </si>
+  <si>
+    <t>10000001373</t>
+  </si>
+  <si>
+    <t>5550000016</t>
+  </si>
+  <si>
+    <t>Renas</t>
+  </si>
+  <si>
+    <t>5550000003</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>Turgut</t>
+  </si>
+  <si>
+    <t>Can</t>
+  </si>
+  <si>
+    <t>10000001374</t>
+  </si>
+  <si>
+    <t>5550000017</t>
+  </si>
+  <si>
+    <t>Niyazi</t>
+  </si>
+  <si>
+    <t>5550000004</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>Merve</t>
+  </si>
+  <si>
+    <t>Işık</t>
+  </si>
+  <si>
+    <t>10000001375</t>
+  </si>
+  <si>
+    <t>5550000018</t>
+  </si>
+  <si>
+    <t>Nupelda</t>
+  </si>
+  <si>
+    <t>5550000005</t>
+  </si>
+  <si>
+    <t>105</t>
+  </si>
+  <si>
+    <t>Ayşe</t>
+  </si>
+  <si>
+    <t>Nesin</t>
+  </si>
+  <si>
+    <t>10000001376</t>
+  </si>
+  <si>
+    <t>5550000019</t>
+  </si>
+  <si>
+    <t>Esmer</t>
+  </si>
+  <si>
+    <t>5550000006</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>Elif</t>
+  </si>
+  <si>
+    <t>Tok</t>
+  </si>
+  <si>
     <t>8-B</t>
   </si>
   <si>
-    <t>ali.kaya@example.com</t>
-  </si>
-  <si>
-    <t>10000001372</t>
-  </si>
-  <si>
-    <t>5550000015</t>
-  </si>
-  <si>
-    <t>Mehmet</t>
-  </si>
-  <si>
-    <t>5550000002</t>
-  </si>
-  <si>
-    <t>veli.kaya@example.com</t>
+    <t>10000001377</t>
+  </si>
+  <si>
+    <t>5550000020</t>
+  </si>
+  <si>
+    <t>Evindar</t>
+  </si>
+  <si>
+    <t>5550000007</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>Umut</t>
+  </si>
+  <si>
+    <t>Anıl</t>
+  </si>
+  <si>
+    <t>10000001378</t>
+  </si>
+  <si>
+    <t>5550000021</t>
+  </si>
+  <si>
+    <t>Murat</t>
+  </si>
+  <si>
+    <t>5550000008</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>Hakan</t>
+  </si>
+  <si>
+    <t>Kal</t>
+  </si>
+  <si>
+    <t>10000001379</t>
+  </si>
+  <si>
+    <t>5550000022</t>
+  </si>
+  <si>
+    <t>Necla</t>
+  </si>
+  <si>
+    <t>5550000009</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>Kader</t>
+  </si>
+  <si>
+    <t>Van</t>
+  </si>
+  <si>
+    <t>10000001380</t>
+  </si>
+  <si>
+    <t>5550000023</t>
+  </si>
+  <si>
+    <t>Mustafa</t>
+  </si>
+  <si>
+    <t>5550000010</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>Yasemin</t>
+  </si>
+  <si>
+    <t>Bingöl</t>
+  </si>
+  <si>
+    <t>10000001381</t>
+  </si>
+  <si>
+    <t>5550000024</t>
+  </si>
+  <si>
+    <t>5550000011</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>Buca</t>
+  </si>
+  <si>
+    <t>10000001382</t>
+  </si>
+  <si>
+    <t>5550000025</t>
+  </si>
+  <si>
+    <t>5550000012</t>
+  </si>
+  <si>
+    <t>112</t>
+  </si>
+  <si>
+    <t>TYT/AYT-A</t>
+  </si>
+  <si>
+    <t>10000001383</t>
+  </si>
+  <si>
+    <t>5550000026</t>
+  </si>
+  <si>
+    <t>5550000013</t>
+  </si>
+  <si>
+    <t>113</t>
+  </si>
+  <si>
+    <t>Tire</t>
+  </si>
+  <si>
+    <t>10000001384</t>
+  </si>
+  <si>
+    <t>5550000027</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>Dal</t>
+  </si>
+  <si>
+    <t>10000001385</t>
+  </si>
+  <si>
+    <t>5550000028</t>
+  </si>
+  <si>
+    <t>115</t>
+  </si>
+  <si>
+    <t>Ön</t>
+  </si>
+  <si>
+    <t>10000001386</t>
+  </si>
+  <si>
+    <t>5550000029</t>
+  </si>
+  <si>
+    <t>116</t>
+  </si>
+  <si>
+    <t>Üst</t>
+  </si>
+  <si>
+    <t>TYT/AYT-B</t>
+  </si>
+  <si>
+    <t>10000001387</t>
+  </si>
+  <si>
+    <t>5550000030</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>Alt</t>
+  </si>
+  <si>
+    <t>10000001388</t>
+  </si>
+  <si>
+    <t>5550000031</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>Alman</t>
+  </si>
+  <si>
+    <t>10000001389</t>
+  </si>
+  <si>
+    <t>5550000032</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>Salla</t>
+  </si>
+  <si>
+    <t>10000001390</t>
+  </si>
+  <si>
+    <t>5550000033</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>Orak</t>
+  </si>
+  <si>
+    <t>10000001391</t>
+  </si>
+  <si>
+    <t>5550000034</t>
   </si>
   <si>
     <t>Alan</t>
@@ -157,10 +469,9 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -169,16 +480,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF14537D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0F766E"/>
+        <fgColor rgb="FFFFF200"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -186,39 +492,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD6DEE8"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD6DEE8"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD6DEE8"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD6DEE8"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -234,60 +516,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="OgrenciAktarimTablosu" displayName="OgrenciAktarimTablosu" ref="A1:O3" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:O3">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-    <filterColumn colId="12" hiddenButton="1"/>
-    <filterColumn colId="13" hiddenButton="1"/>
-    <filterColumn colId="14" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="15">
-    <tableColumn id="1" name="okul_no" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="ad" totalsRowFunction="none"/>
-    <tableColumn id="3" name="soyad" totalsRowFunction="none"/>
-    <tableColumn id="4" name="sinif" totalsRowFunction="none"/>
-    <tableColumn id="5" name="email" totalsRowFunction="none"/>
-    <tableColumn id="6" name="tc_kimlik_no" totalsRowFunction="none"/>
-    <tableColumn id="7" name="telefon" totalsRowFunction="none"/>
-    <tableColumn id="8" name="veli_ad" totalsRowFunction="none"/>
-    <tableColumn id="9" name="veli_soyad" totalsRowFunction="none"/>
-    <tableColumn id="10" name="veli_telefon" totalsRowFunction="none"/>
-    <tableColumn id="11" name="veli_email" totalsRowFunction="none"/>
-    <tableColumn id="12" name="veli_finans" totalsRowFunction="none"/>
-    <tableColumn id="13" name="veli_sms" totalsRowFunction="none"/>
-    <tableColumn id="14" name="veli_duyuru" totalsRowFunction="none"/>
-    <tableColumn id="15" name="veli_destek" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="OgrenciSecenekleri" displayName="OgrenciSecenekleri" ref="A1:B8" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:B8">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Alan" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Kabul edilen değerler" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -612,167 +840,1057 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="23" customWidth="1"/>
-    <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="15" width="13" customWidth="1"/>
+    <col min="1" max="4" width="12" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14" style="1" customWidth="1"/>
+    <col min="7" max="9" width="12" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14" style="1" customWidth="1"/>
+    <col min="11" max="11" width="23" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="1" customWidth="1"/>
+    <col min="14" max="15" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="L2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="L3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="2" t="s">
+      <c r="F4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="I13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O22" s="1" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -781,79 +1899,76 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="82" customWidth="1"/>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>38</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>39</v>
+      <c r="B2" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>40</v>
+      <c r="B3" s="1" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>41</v>
+      <c r="B4" s="1" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>42</v>
+      <c r="B5" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>42</v>
+      <c r="B6" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>42</v>
+      <c r="B7" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>42</v>
+      <c r="B8" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix student import template tc values
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
@@ -128,7 +128,7 @@
     <t>Saya</t>
   </si>
   <si>
-    <t>10000001373</t>
+    <t>10000002508</t>
   </si>
   <si>
     <t>5550000016</t>
@@ -149,7 +149,7 @@
     <t>Can</t>
   </si>
   <si>
-    <t>10000001374</t>
+    <t>10000002676</t>
   </si>
   <si>
     <t>5550000017</t>
@@ -170,7 +170,7 @@
     <t>Işık</t>
   </si>
   <si>
-    <t>10000001375</t>
+    <t>10000002744</t>
   </si>
   <si>
     <t>5550000018</t>
@@ -191,7 +191,7 @@
     <t>Nesin</t>
   </si>
   <si>
-    <t>10000001376</t>
+    <t>10000002812</t>
   </si>
   <si>
     <t>5550000019</t>
@@ -215,7 +215,7 @@
     <t>8-B</t>
   </si>
   <si>
-    <t>10000001377</t>
+    <t>10000002980</t>
   </si>
   <si>
     <t>5550000020</t>
@@ -236,7 +236,7 @@
     <t>Anıl</t>
   </si>
   <si>
-    <t>10000001378</t>
+    <t>10000003048</t>
   </si>
   <si>
     <t>5550000021</t>
@@ -257,7 +257,7 @@
     <t>Kal</t>
   </si>
   <si>
-    <t>10000001379</t>
+    <t>10000003116</t>
   </si>
   <si>
     <t>5550000022</t>
@@ -278,7 +278,7 @@
     <t>Van</t>
   </si>
   <si>
-    <t>10000001380</t>
+    <t>10000003284</t>
   </si>
   <si>
     <t>5550000023</t>
@@ -299,7 +299,7 @@
     <t>Bingöl</t>
   </si>
   <si>
-    <t>10000001381</t>
+    <t>10000003352</t>
   </si>
   <si>
     <t>5550000024</t>
@@ -314,7 +314,7 @@
     <t>Buca</t>
   </si>
   <si>
-    <t>10000001382</t>
+    <t>10000003420</t>
   </si>
   <si>
     <t>5550000025</t>
@@ -329,7 +329,7 @@
     <t>TYT/AYT-A</t>
   </si>
   <si>
-    <t>10000001383</t>
+    <t>10000003598</t>
   </si>
   <si>
     <t>5550000026</t>
@@ -344,7 +344,7 @@
     <t>Tire</t>
   </si>
   <si>
-    <t>10000001384</t>
+    <t>10000003666</t>
   </si>
   <si>
     <t>5550000027</t>
@@ -356,7 +356,7 @@
     <t>Dal</t>
   </si>
   <si>
-    <t>10000001385</t>
+    <t>10000003734</t>
   </si>
   <si>
     <t>5550000028</t>
@@ -368,7 +368,7 @@
     <t>Ön</t>
   </si>
   <si>
-    <t>10000001386</t>
+    <t>10000003802</t>
   </si>
   <si>
     <t>5550000029</t>
@@ -383,7 +383,7 @@
     <t>TYT/AYT-B</t>
   </si>
   <si>
-    <t>10000001387</t>
+    <t>10000003970</t>
   </si>
   <si>
     <t>5550000030</t>
@@ -395,7 +395,7 @@
     <t>Alt</t>
   </si>
   <si>
-    <t>10000001388</t>
+    <t>10000004038</t>
   </si>
   <si>
     <t>5550000031</t>
@@ -407,7 +407,7 @@
     <t>Alman</t>
   </si>
   <si>
-    <t>10000001389</t>
+    <t>10000004106</t>
   </si>
   <si>
     <t>5550000032</t>
@@ -419,7 +419,7 @@
     <t>Salla</t>
   </si>
   <si>
-    <t>10000001390</t>
+    <t>10000004274</t>
   </si>
   <si>
     <t>5550000033</t>
@@ -431,7 +431,7 @@
     <t>Orak</t>
   </si>
   <si>
-    <t>10000001391</t>
+    <t>10000004342</t>
   </si>
   <si>
     <t>5550000034</t>
@@ -1890,7 +1890,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1969,6 +1969,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: refresh import templates and align import-service behavior
Student template drops the permission columns and adds
veli_tc_kimlik_no; teacher template adds optional atanacak_sinif and
ders columns; new kazanim-aktarim-sablonu.xlsx for learning outcome
import. Fixture contract pins the new headers. Teacher import errors
now mask national ids and omit raw phone values like the student
import. Demo fixtures fall back to built-in rows when the header-only
workbooks carry no data.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogrenci-aktarim-sablonu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="27">
   <si>
     <t>okul_no</t>
   </si>
@@ -45,16 +45,7 @@
     <t>veli_telefon</t>
   </si>
   <si>
-    <t>veli_finans</t>
-  </si>
-  <si>
-    <t>veli_sms</t>
-  </si>
-  <si>
-    <t>veli_duyuru</t>
-  </si>
-  <si>
-    <t>veli_destek</t>
+    <t>veli_tc_kimlik_no</t>
   </si>
   <si>
     <t>alan</t>
@@ -63,58 +54,46 @@
     <t>aciklama</t>
   </si>
   <si>
-    <t>Kurum icindeki ogrenci numarasi. Bos birakilabilir; doluysa benzersiz olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogrenci adi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogrenci soyadi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Sistemde tanimli sinif adi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogrenci e-postasi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogrenci TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogrenci cep telefonu. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Veli adi. Veli baglantisi kurulacaksa soyad ve telefonla birlikte doldurun.</t>
-  </si>
-  <si>
-    <t>Veli soyadi.</t>
-  </si>
-  <si>
-    <t>Veli cep telefonu. Veli TC girildiyse zorunludur.</t>
-  </si>
-  <si>
-    <t>Veli finans bilgilerini gorebilir mi?</t>
-  </si>
-  <si>
-    <t>Veli SMS alabilir mi?</t>
-  </si>
-  <si>
-    <t>Veli duyuru alabilir mi?</t>
-  </si>
-  <si>
-    <t>Veli destek talebi acabilir mi?</t>
-  </si>
-  <si>
-    <t>gecerli_degerler</t>
-  </si>
-  <si>
-    <t>11 haneli gecerli TC kimlik no</t>
-  </si>
-  <si>
-    <t>+905XXXXXXXXX veya 05XXXXXXXXX</t>
-  </si>
-  <si>
-    <t>evet, hayir, true, false, 1, 0</t>
+    <t>Opsiyonel okul numarası. Aynı kurum içinde tekil tutulur.</t>
+  </si>
+  <si>
+    <t>Zorunlu öğrenci adı.</t>
+  </si>
+  <si>
+    <t>Zorunlu öğrenci soyadı.</t>
+  </si>
+  <si>
+    <t>Opsiyonel sınıf adı. Örn. 8-A.</t>
+  </si>
+  <si>
+    <t>Opsiyonel öğrenci e-posta adresi.</t>
+  </si>
+  <si>
+    <t>Opsiyonel öğrenci TC kimlik numarası.</t>
+  </si>
+  <si>
+    <t>Opsiyonel öğrenci telefonu.</t>
+  </si>
+  <si>
+    <t>Opsiyonel veli adı.</t>
+  </si>
+  <si>
+    <t>Opsiyonel veli soyadı.</t>
+  </si>
+  <si>
+    <t>Opsiyonel veli telefonu.</t>
+  </si>
+  <si>
+    <t>Opsiyonel veli TC kimlik numarası. Veli izinleri SMS, duyuru, finans ve destek için otomatik açık gelir.</t>
+  </si>
+  <si>
+    <t>secenek</t>
+  </si>
+  <si>
+    <t>8-A</t>
+  </si>
+  <si>
+    <t>05550000000</t>
   </si>
 </sst>
 </file>
@@ -153,17 +132,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,19 +474,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="14" width="15" customWidth="1"/>
+    <col min="1" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -549,18 +515,8 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -568,131 +524,107 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="2" max="2" width="88" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -703,75 +635,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>33</v>
+      <c r="B3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>